<commit_message>
Step 1: adopt hysteresis + gap bridging as defaults
THRESHOLD_MODE="hysteresis", HYSTERESIS_LOW_FRACTION=0.75 and
GAP_BRIDGING=True are now defaults, on the Phase 2 guard comparison plus
the visual crop check confirming added connections follow real dim
threads. Of eight settings tried this was inside both pre-declared guards
on tuning AND held-out (1.13x length vs a 1.20x limit, 2.13x loops vs
max(1.5x, +50)) while cutting components per 10,000 skeleton px from 225
to 169.

THE 543-2 REFERENCE CHECK CHANGES: 37.00 / 29.43 (old) -> 62.33 / 27.41
with 21 bridges (new). Both recorded in PROGRESS.md; the old path stays
reproducible via --threshold-mode multiotsu_low and omitting
--gap-bridging.

The +68% jump in edge count is expected and is why Phase 4 recommended
against edge count as a primary outcome -- it is the most
segmentation-sensitive metric measured. Per-field metrics and roots/cell
moved ~11-13% over the same change.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/canaliculi/543-2/measurements.xlsx
+++ b/results/canaliculi/543-2/measurements.xlsx
@@ -531,13 +531,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>37</v>
+        <v>62.3333</v>
       </c>
       <c r="C7" t="n">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="D7" t="n">
-        <v>26.4953</v>
+        <v>44.9188</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -555,13 +555,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1072.3365</v>
+        <v>1687.3328</v>
       </c>
       <c r="C8" t="n">
-        <v>858.7016</v>
+        <v>1266.4158</v>
       </c>
       <c r="D8" t="n">
-        <v>781.1651000000001</v>
+        <v>1263.5954</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -579,13 +579,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>29.4324</v>
+        <v>27.4088</v>
       </c>
       <c r="C9" t="n">
-        <v>28.9201</v>
+        <v>28.085</v>
       </c>
       <c r="D9" t="n">
-        <v>6.2832</v>
+        <v>4.2017</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>40240</v>
+        <v>45785</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.03928763</v>
+        <v>0.04470139</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>452</v>
+        <v>681</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.0004413</v>
+        <v>0.00066488</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>756</v>
+        <v>673</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>53.2275</v>
+        <v>68.0312</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -847,13 +847,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C2" t="n">
-        <v>2078.8368</v>
+        <v>1615.5454</v>
       </c>
       <c r="D2" t="n">
-        <v>25.0462</v>
+        <v>22.1308</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -869,13 +869,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>53</v>
+        <v>146</v>
       </c>
       <c r="C3" t="n">
-        <v>1498.4499</v>
+        <v>3672.5811</v>
       </c>
       <c r="D3" t="n">
-        <v>28.2726</v>
+        <v>25.1547</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -891,13 +891,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" t="n">
-        <v>987.0631</v>
+        <v>1009.4478</v>
       </c>
       <c r="D4" t="n">
-        <v>26.6774</v>
+        <v>28.8414</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -913,13 +913,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C5" t="n">
-        <v>363.9361</v>
+        <v>1016.0925</v>
       </c>
       <c r="D5" t="n">
-        <v>17.3303</v>
+        <v>19.5402</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -935,13 +935,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C6" t="n">
-        <v>240.2082</v>
+        <v>509.0021</v>
       </c>
       <c r="D6" t="n">
-        <v>40.0347</v>
+        <v>28.2779</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -957,13 +957,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="C7" t="n">
-        <v>2145.1677</v>
+        <v>1516.7392</v>
       </c>
       <c r="D7" t="n">
-        <v>30.6453</v>
+        <v>30.3348</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -979,13 +979,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C8" t="n">
-        <v>330.1787</v>
+        <v>352.664</v>
       </c>
       <c r="D8" t="n">
-        <v>27.5149</v>
+        <v>35.2664</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -1001,13 +1001,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>57</v>
+        <v>103</v>
       </c>
       <c r="C9" t="n">
-        <v>1685.3616</v>
+        <v>3205.0836</v>
       </c>
       <c r="D9" t="n">
-        <v>29.5677</v>
+        <v>31.1173</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -1023,13 +1023,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="C10" t="n">
-        <v>402.3919</v>
+        <v>568.7595</v>
       </c>
       <c r="D10" t="n">
-        <v>33.5327</v>
+        <v>25.8527</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -1045,13 +1045,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C11" t="n">
-        <v>297.865</v>
+        <v>826.2397</v>
       </c>
       <c r="D11" t="n">
-        <v>22.9127</v>
+        <v>25.0376</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -1067,13 +1067,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>60</v>
+        <v>134</v>
       </c>
       <c r="C12" t="n">
-        <v>2108.2388</v>
+        <v>3947.6004</v>
       </c>
       <c r="D12" t="n">
-        <v>35.1373</v>
+        <v>29.4597</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -1089,13 +1089,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>20</v>
+        <v>72</v>
       </c>
       <c r="C13" t="n">
-        <v>730.3402</v>
+        <v>2008.2388</v>
       </c>
       <c r="D13" t="n">
-        <v>36.517</v>
+        <v>27.8922</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>

</xml_diff>